<commit_message>
fix(extract): AUTO_POST raggiungibile e eval onesta
Ritarata la confidenza (0,98 deterministica, 0,99 accordo) così un ordine
pulito supera auto_post_min_score 0,97, lasciata invariata la soglia §7.1.
CUS-03 ignora ship_to solo-nome, EXT-02 confronta 24.0/$/USD in modo
tollerante, buyer_item_code assente non ha più confidenza 0.

Errore silenzioso = AUTO_POST con almeno un campo sbagliato (testata,
codice/qty/UoM/prezzo, righe extra/mancanti, allucinazioni). make eval
fissa seed/modello/parametri, scrive eval_results.json ordine per ordine,
carica i numeri «prima» da git show 380c7bb e ripete la run senza LLM.

Corrette le date Excel e DATE_FORMAT; cinque template email fuori dalle
regex attuali. PDF esclusi da questo campione.

Co-authored-by: RBossio <RBossio@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/synthetic/documents/eml/order_094_APE-01093.xlsx
+++ b/synthetic/documents/eml/order_094_APE-01093.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Purchase Order" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Purchase Order" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -511,229 +511,212 @@
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Delivery Date:</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>Line</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>Item Code</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="D9" s="3" t="inlineStr">
         <is>
           <t>Quantity</t>
         </is>
       </c>
-      <c r="E8" s="3" t="inlineStr">
+      <c r="E9" s="3" t="inlineStr">
         <is>
           <t>UoM</t>
         </is>
       </c>
-      <c r="F8" s="3" t="inlineStr">
+      <c r="F9" s="3" t="inlineStr">
         <is>
           <t>Unit Price</t>
         </is>
       </c>
-      <c r="G8" s="3" t="inlineStr">
+      <c r="G9" s="3" t="inlineStr">
         <is>
           <t>Amount</t>
         </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>SUMMIT-LUB-2596</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>Multi-Purpose Grease (SYNTHETIC)</t>
-        </is>
-      </c>
-      <c r="D9" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="E9" s="4" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="F9" s="4" t="n">
-        <v>73.89</v>
-      </c>
-      <c r="G9" s="4" t="n">
-        <v>1773.36</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>SUMMIT-TOO-2055</t>
+          <t>SUMMIT-LUB-2596</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Utility Blade Standard (SYNTHETIC)</t>
+          <t>Multi-Purpose Grease (SYNTHETIC)</t>
         </is>
       </c>
       <c r="D10" s="4" t="n">
-        <v>1</v>
+        <v>24</v>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>PK</t>
+          <t>CS</t>
         </is>
       </c>
       <c r="F10" s="4" t="n">
-        <v>7.32</v>
+        <v>73.89</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>7.32</v>
+        <v>1773.36</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>SUMMIT-FAS-3679</t>
+          <t>SUMMIT-TOO-2055</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Hex Cap Screw 3/8-16 x 1-1/2 Grade 5 Zinc (SYNTHETIC)</t>
+          <t>Utility Blade Standard (SYNTHETIC)</t>
         </is>
       </c>
       <c r="D11" s="4" t="n">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>BX</t>
+          <t>PK</t>
         </is>
       </c>
       <c r="F11" s="4" t="n">
-        <v>27.99</v>
+        <v>7.32</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>671.76</v>
+        <v>7.32</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>PKG-BBW-105</t>
+          <t>SUMMIT-FAS-3679</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Bubble Wrap 12in (SYNTHETIC)</t>
+          <t>Hex Cap Screw 3/8-16 x 1-1/2 Grade 5 Zinc (SYNTHETIC)</t>
         </is>
       </c>
       <c r="D12" s="4" t="n">
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>RO</t>
+          <t>BX</t>
         </is>
       </c>
       <c r="F12" s="4" t="n">
-        <v>51.78</v>
+        <v>27.99</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>103.56</v>
+        <v>671.76</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>SUMMIT-JAN-5714</t>
+          <t>PKG-BBW-105</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Glass Cleaner RTU (SYNTHETIC)</t>
+          <t>Bubble Wrap 12in (SYNTHETIC)</t>
         </is>
       </c>
       <c r="D13" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>CS</t>
+          <t>RO</t>
         </is>
       </c>
       <c r="F13" s="4" t="n">
-        <v>29.19</v>
+        <v>51.78</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>87.56999999999999</v>
+        <v>103.56</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>PKG-BBW-005</t>
+          <t>SUMMIT-JAN-5714</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Bubble Wrap 12in (SYNTHETIC)</t>
+          <t>Glass Cleaner RTU (SYNTHETIC)</t>
         </is>
       </c>
       <c r="D14" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>RO</t>
+          <t>CS</t>
         </is>
       </c>
       <c r="F14" s="4" t="n">
-        <v>37.59</v>
+        <v>29.19</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>187.95</v>
+        <v>87.56999999999999</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>PPE-N95-288</t>
+          <t>PKG-BBW-005</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>N95 Respirator (SYNTHETIC)</t>
+          <t>Bubble Wrap 12in (SYNTHETIC)</t>
         </is>
       </c>
       <c r="D15" s="4" t="n">
@@ -741,42 +724,71 @@
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>BX</t>
+          <t>RO</t>
         </is>
       </c>
       <c r="F15" s="4" t="n">
-        <v>37.47</v>
+        <v>37.59</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>187.35</v>
+        <v>187.95</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>PPE-N95-288</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>N95 Respirator (SYNTHETIC)</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>BX</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="n">
+        <v>37.47</v>
+      </c>
+      <c r="G16" s="4" t="n">
+        <v>187.35</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="B16" s="4" t="inlineStr">
+      <c r="B17" s="4" t="inlineStr">
         <is>
           <t>SUMMIT-ELE-0244</t>
         </is>
       </c>
-      <c r="C16" s="4" t="inlineStr">
+      <c r="C17" s="4" t="inlineStr">
         <is>
           <t>Wire Nut 3/4-10 {color} (SYNTHETIC)</t>
         </is>
       </c>
-      <c r="D16" s="4" t="n">
+      <c r="D17" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="E16" s="4" t="inlineStr">
+      <c r="E17" s="4" t="inlineStr">
         <is>
           <t>BX</t>
         </is>
       </c>
-      <c r="F16" s="4" t="n">
+      <c r="F17" s="4" t="n">
         <v>20.66</v>
       </c>
-      <c r="G16" s="4" t="n">
+      <c r="G17" s="4" t="n">
         <v>41.32</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Estrazione deterministica, eval riproducibile e confidenza tarata (#18)
Preprocessor deterministico Excel/PDF, confidenza tarata, regole EXT/QTY/CUS più severe, make eval riproducibile (seed 42, 50 ordini, senza PDF).

Verificato su a2bb197: pytest 1050 passed, ruff 0.4.4 e mypy 1.10 verdi, CI lint+test verdi.
Eval senza LLM: AUTO_POST 29/50, errori silenziosi 0/29, testata 83,0%, righe 44,4% (prima su aea6f9b: 25,0% / 41,5%, AUTO_POST 0/50). Numeri su dati sintetici.
CatalogMatcher.allowlist_synthetic=False di default, True solo in make eval. Valuta assente: anagrafica (0,97, fonte catalog) o default 0,50 -> REVIEW. QTY-02 per quantità x100; cliente solo da xref -> REVIEW. UI: 10 ordini demo, ordine non risolto non crea bozza.
</commit_message>
<xml_diff>
--- a/synthetic/documents/eml/order_094_APE-01093.xlsx
+++ b/synthetic/documents/eml/order_094_APE-01093.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Purchase Order" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Purchase Order" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -511,229 +511,212 @@
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Delivery Date:</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>Line</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>Item Code</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="D9" s="3" t="inlineStr">
         <is>
           <t>Quantity</t>
         </is>
       </c>
-      <c r="E8" s="3" t="inlineStr">
+      <c r="E9" s="3" t="inlineStr">
         <is>
           <t>UoM</t>
         </is>
       </c>
-      <c r="F8" s="3" t="inlineStr">
+      <c r="F9" s="3" t="inlineStr">
         <is>
           <t>Unit Price</t>
         </is>
       </c>
-      <c r="G8" s="3" t="inlineStr">
+      <c r="G9" s="3" t="inlineStr">
         <is>
           <t>Amount</t>
         </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>SUMMIT-LUB-2596</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>Multi-Purpose Grease (SYNTHETIC)</t>
-        </is>
-      </c>
-      <c r="D9" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="E9" s="4" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="F9" s="4" t="n">
-        <v>73.89</v>
-      </c>
-      <c r="G9" s="4" t="n">
-        <v>1773.36</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>SUMMIT-TOO-2055</t>
+          <t>SUMMIT-LUB-2596</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Utility Blade Standard (SYNTHETIC)</t>
+          <t>Multi-Purpose Grease (SYNTHETIC)</t>
         </is>
       </c>
       <c r="D10" s="4" t="n">
-        <v>1</v>
+        <v>24</v>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>PK</t>
+          <t>CS</t>
         </is>
       </c>
       <c r="F10" s="4" t="n">
-        <v>7.32</v>
+        <v>73.89</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>7.32</v>
+        <v>1773.36</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>SUMMIT-FAS-3679</t>
+          <t>SUMMIT-TOO-2055</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Hex Cap Screw 3/8-16 x 1-1/2 Grade 5 Zinc (SYNTHETIC)</t>
+          <t>Utility Blade Standard (SYNTHETIC)</t>
         </is>
       </c>
       <c r="D11" s="4" t="n">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>BX</t>
+          <t>PK</t>
         </is>
       </c>
       <c r="F11" s="4" t="n">
-        <v>27.99</v>
+        <v>7.32</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>671.76</v>
+        <v>7.32</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>PKG-BBW-105</t>
+          <t>SUMMIT-FAS-3679</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Bubble Wrap 12in (SYNTHETIC)</t>
+          <t>Hex Cap Screw 3/8-16 x 1-1/2 Grade 5 Zinc (SYNTHETIC)</t>
         </is>
       </c>
       <c r="D12" s="4" t="n">
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>RO</t>
+          <t>BX</t>
         </is>
       </c>
       <c r="F12" s="4" t="n">
-        <v>51.78</v>
+        <v>27.99</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>103.56</v>
+        <v>671.76</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>SUMMIT-JAN-5714</t>
+          <t>PKG-BBW-105</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Glass Cleaner RTU (SYNTHETIC)</t>
+          <t>Bubble Wrap 12in (SYNTHETIC)</t>
         </is>
       </c>
       <c r="D13" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>CS</t>
+          <t>RO</t>
         </is>
       </c>
       <c r="F13" s="4" t="n">
-        <v>29.19</v>
+        <v>51.78</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>87.56999999999999</v>
+        <v>103.56</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>PKG-BBW-005</t>
+          <t>SUMMIT-JAN-5714</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Bubble Wrap 12in (SYNTHETIC)</t>
+          <t>Glass Cleaner RTU (SYNTHETIC)</t>
         </is>
       </c>
       <c r="D14" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>RO</t>
+          <t>CS</t>
         </is>
       </c>
       <c r="F14" s="4" t="n">
-        <v>37.59</v>
+        <v>29.19</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>187.95</v>
+        <v>87.56999999999999</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>PPE-N95-288</t>
+          <t>PKG-BBW-005</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>N95 Respirator (SYNTHETIC)</t>
+          <t>Bubble Wrap 12in (SYNTHETIC)</t>
         </is>
       </c>
       <c r="D15" s="4" t="n">
@@ -741,42 +724,71 @@
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>BX</t>
+          <t>RO</t>
         </is>
       </c>
       <c r="F15" s="4" t="n">
-        <v>37.47</v>
+        <v>37.59</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>187.35</v>
+        <v>187.95</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>PPE-N95-288</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>N95 Respirator (SYNTHETIC)</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>BX</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="n">
+        <v>37.47</v>
+      </c>
+      <c r="G16" s="4" t="n">
+        <v>187.35</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="B16" s="4" t="inlineStr">
+      <c r="B17" s="4" t="inlineStr">
         <is>
           <t>SUMMIT-ELE-0244</t>
         </is>
       </c>
-      <c r="C16" s="4" t="inlineStr">
+      <c r="C17" s="4" t="inlineStr">
         <is>
           <t>Wire Nut 3/4-10 {color} (SYNTHETIC)</t>
         </is>
       </c>
-      <c r="D16" s="4" t="n">
+      <c r="D17" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="E16" s="4" t="inlineStr">
+      <c r="E17" s="4" t="inlineStr">
         <is>
           <t>BX</t>
         </is>
       </c>
-      <c r="F16" s="4" t="n">
+      <c r="F17" s="4" t="n">
         <v>20.66</v>
       </c>
-      <c r="G16" s="4" t="n">
+      <c r="G17" s="4" t="n">
         <v>41.32</v>
       </c>
     </row>

</xml_diff>